<commit_message>
feat: add registration flow, enable API sync, personalize home screen
- Enable API sync pointing to http://agent.home/api (30min interval)
- Set default routes to /template/registration
- Add registration template with phone_number-based flow
- Add personalized greeting and login count to home screen
- Add registration template to sheet metadata
</commit_message>
<xml_diff>
--- a/sheets/my_website.xlsx
+++ b/sheets/my_website.xlsx
@@ -13,6 +13,7 @@
     <sheet name="blog_list" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="contact_page" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="app_menu" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="registration" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +534,23 @@
         </is>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>released</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>registration</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>released</t>
         </is>
@@ -549,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,22 +610,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hero_title</t>
+          <t>greeting</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Welcome to My Website</t>
+          <t>Hello, @fields.user_name!</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Main hero heading</t>
+          <t>Personalized greeting</t>
         </is>
       </c>
     </row>
@@ -619,56 +637,51 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hero_subtitle</t>
+          <t>login_count</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A simple app built with Open App Builder. Explore the sections below.</t>
+          <t>You have been logged in @fields.login_count times</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>btn_about</t>
+          <t>hero_title</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>About Us</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>click | go_to:about_page</t>
+          <t>Welcome to My Website</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Main hero heading</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>btn_blog</t>
+          <t>hero_subtitle</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Read Our Blog</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>click | go_to:blog_list</t>
+          <t>A simple app built with Open App Builder. Explore the sections below.</t>
         </is>
       </c>
     </row>
@@ -680,15 +693,59 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>btn_about</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>About Us</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>click | go_to:about_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>btn_blog</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Read Our Blog</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>click | go_to:blog_list</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>btn_contact</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Contact Us</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>click | go_to:contact_page</t>
         </is>
@@ -1427,4 +1484,197 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>action_list</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>parameter_list</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>reg_title</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>!@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>text_box</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>name_input</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>placeholder: Your name</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>!@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>text_box</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>phone_input</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>placeholder: Phone number</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>!@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>btn_register</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>click | set_field : user_name : @local.name_input ;; click | set_field : phone_number : @local.phone_input ;; click | go_to : home_screen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>!@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>reg_welcome_back</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Welcome back, @fields.user_name!</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>btn_go_home</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Continue</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>click | go_to : home_screen</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>@fields.phone_number</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add greeting header card with progress bar on home screen
Replace plain text greeting/login rows with an Ionic card component
showing the user's name, login count, and a 50% progress bar.

Signed-off-by: Xuewei Niu <justxuewei@apache.org>
</commit_message>
<xml_diff>
--- a/sheets/my_website.xlsx
+++ b/sheets/my_website.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,78 +610,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>html</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>greeting</t>
+          <t>header_card</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello, @fields.user_name!</t>
+          <t>&lt;ion-card&gt;&lt;ion-card-header&gt;&lt;ion-card-title&gt;Hello, @fields.user_name!&lt;/ion-card-title&gt;&lt;ion-card-subtitle&gt;You have logged in @fields.login_count times&lt;/ion-card-subtitle&gt;&lt;/ion-card-header&gt;&lt;ion-card-content&gt;&lt;p style="margin-bottom: 8px; font-size: 0.875rem; color: var(--ion-color-medium)"&gt;Your progress&lt;/p&gt;&lt;ion-progress-bar value="0.5"&gt;&lt;/ion-progress-bar&gt;&lt;p style="margin-top: 4px; font-size: 0.75rem; color: var(--ion-color-medium); text-align: right"&gt;50%&lt;/p&gt;&lt;/ion-card-content&gt;&lt;/ion-card&gt;</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Personalized greeting</t>
+          <t>Greeting card with progress</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>login_count</t>
+          <t>hero_title</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>You have been logged in @fields.login_count times</t>
+          <t>Welcome to ParentingApp</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Main hero heading</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>hero_title</t>
+          <t>hero_subtitle</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Welcome to My Website</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Main hero heading</t>
+          <t>A simple app built with Open App Builder. Explore the sections below.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>button</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hero_subtitle</t>
+          <t>btn_about</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A simple app built with Open App Builder. Explore the sections below.</t>
+          <t>About Us</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>click | go_to:about_page</t>
         </is>
       </c>
     </row>
@@ -693,17 +698,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>btn_about</t>
+          <t>btn_blog</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>About Us</t>
+          <t>Read Our Blog</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>click | go_to:about_page</t>
+          <t>click | go_to:blog_list</t>
         </is>
       </c>
     </row>
@@ -715,37 +720,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>btn_blog</t>
+          <t>btn_contact</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Read Our Blog</t>
+          <t>Contact Us</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
-        <is>
-          <t>click | go_to:blog_list</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>button</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>btn_contact</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Contact Us</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
         <is>
           <t>click | go_to:contact_page</t>
         </is>

</xml_diff>

<commit_message>
content: update title to ParentingApp and update blog posts
Signed-off-by: Xuewei Niu <justxuewei@apache.org>
</commit_message>
<xml_diff>
--- a/sheets/my_website.xlsx
+++ b/sheets/my_website.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -985,17 +985,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>post1_title</t>
+          <t>post4_title</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Getting Started with Open App Builder</t>
+          <t>Getting start with ParentingApp built by RUC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Blog post 1</t>
+          <t>Blog post 4</t>
         </is>
       </c>
     </row>
@@ -1007,12 +1007,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>post1_date</t>
+          <t>post4_date</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>March 20, 2026</t>
+          <t>March 29, 2026</t>
         </is>
       </c>
     </row>
@@ -1024,12 +1024,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>post1_excerpt</t>
+          <t>post4_excerpt</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Learn how to set up your first app in minutes using spreadsheets as your content source.</t>
+          <t>Discover how the ParentingApp, built by RUC, empowers parents with tools to track, learn, and grow alongside their children.</t>
         </is>
       </c>
     </row>
@@ -1041,17 +1041,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>post2_title</t>
+          <t>post3_title</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Why Content-First Design Matters</t>
+          <t>Deploying to a VPS with Nginx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Blog post 2</t>
+          <t>Blog post 3</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1063,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>post2_date</t>
+          <t>post3_date</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>March 25, 2026</t>
+          <t>March 28, 2026</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>post2_excerpt</t>
+          <t>post3_excerpt</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Discover how separating content from code allows non-developers to shape the user experience.</t>
+          <t>A step-by-step guide to hosting your app on Ubuntu with nginx — no Firebase required.</t>
         </is>
       </c>
     </row>
@@ -1097,17 +1097,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>post3_title</t>
+          <t>post2_title</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Deploying to a VPS with Nginx</t>
+          <t>Why Content-First Design Matters</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Blog post 3</t>
+          <t>Blog post 2</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1119,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>post3_date</t>
+          <t>post2_date</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>March 28, 2026</t>
+          <t>March 25, 2026</t>
         </is>
       </c>
     </row>
@@ -1136,32 +1136,88 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>post3_excerpt</t>
+          <t>post2_excerpt</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A step-by-step guide to hosting your app on Ubuntu with nginx — no Firebase required.</t>
+          <t>Discover how separating content from code allows non-developers to shape the user experience.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>post1_title</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Getting Started with Open App Builder</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Blog post 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>post1_date</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>March 20, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>post1_excerpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Learn how to set up your first app in minutes using spreadsheets as your content source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>button</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>btn_back</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>← Back to Home</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>click | go_to:home_screen</t>
         </is>

</xml_diff>